<commit_message>
Updated all test cases and files
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Vehicle.xlsx
+++ b/src/test/resources/testdata/Vehicle.xlsx
@@ -7,12 +7,13 @@
   </bookViews>
   <sheets>
     <sheet name="HondaBikesUnder4Lakhs" r:id="rId3" sheetId="1"/>
+    <sheet name="CarsUnder4Lakh" r:id="rId4" sheetId="2"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
   <si>
     <t>Bike Name</t>
   </si>
@@ -81,6 +82,42 @@
   </si>
   <si>
     <t>Rs. 79,000</t>
+  </si>
+  <si>
+    <t>Car Name</t>
+  </si>
+  <si>
+    <t>Price</t>
+  </si>
+  <si>
+    <t>Maruti Wagon R VXI Minor</t>
+  </si>
+  <si>
+    <t>Rs. 2.00 Lakh</t>
+  </si>
+  <si>
+    <t>Honda Brio S MT</t>
+  </si>
+  <si>
+    <t>Rs. 3.95 Lakh</t>
+  </si>
+  <si>
+    <t>62 Used Honda City</t>
+  </si>
+  <si>
+    <t>Rs. 1.85 Lakh</t>
+  </si>
+  <si>
+    <t>50 Used Kia Seltos</t>
+  </si>
+  <si>
+    <t>Rs. 3.69 Lakh</t>
+  </si>
+  <si>
+    <t>48 Used Hyundai Creta</t>
+  </si>
+  <si>
+    <t>Rs. 3.45 Lakh</t>
   </si>
 </sst>
 </file>
@@ -241,4 +278,62 @@
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B1" t="s" s="0">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>25</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>27</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>29</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>31</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
TC_6 and TC_9 added
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Vehicle.xlsx
+++ b/src/test/resources/testdata/Vehicle.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="31">
   <si>
     <t>Bike Name</t>
   </si>
@@ -90,34 +90,22 @@
     <t>Price</t>
   </si>
   <si>
-    <t>Maruti Wagon R VXI Minor</t>
-  </si>
-  <si>
-    <t>Rs. 2.00 Lakh</t>
-  </si>
-  <si>
-    <t>Honda Brio S MT</t>
-  </si>
-  <si>
-    <t>Rs. 3.95 Lakh</t>
-  </si>
-  <si>
-    <t>62 Used Honda City</t>
-  </si>
-  <si>
-    <t>Rs. 1.85 Lakh</t>
-  </si>
-  <si>
-    <t>50 Used Kia Seltos</t>
-  </si>
-  <si>
-    <t>Rs. 3.69 Lakh</t>
-  </si>
-  <si>
-    <t>48 Used Hyundai Creta</t>
-  </si>
-  <si>
-    <t>Rs. 3.45 Lakh</t>
+    <t>Hyundai Grand i10 1.2 Kappa Asta</t>
+  </si>
+  <si>
+    <t>Rs. 3.18 Lakh</t>
+  </si>
+  <si>
+    <t>Hyundai i10 Magna 1.1</t>
+  </si>
+  <si>
+    <t>Rs. 3.05 Lakh</t>
+  </si>
+  <si>
+    <t>41 Used Hyundai Creta</t>
+  </si>
+  <si>
+    <t>Rs. 3.79 Lakh</t>
   </si>
 </sst>
 </file>
@@ -282,7 +270,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -317,22 +305,6 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>33</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>34</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
TC_10 and TC_11 added
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Vehicle.xlsx
+++ b/src/test/resources/testdata/Vehicle.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="31">
   <si>
     <t>Bike Name</t>
   </si>
@@ -90,34 +90,22 @@
     <t>Price</t>
   </si>
   <si>
-    <t>Maruti Wagon R VXI Minor</t>
-  </si>
-  <si>
-    <t>Rs. 2.00 Lakh</t>
-  </si>
-  <si>
-    <t>Honda Brio S MT</t>
-  </si>
-  <si>
-    <t>Rs. 3.95 Lakh</t>
-  </si>
-  <si>
-    <t>62 Used Honda City</t>
-  </si>
-  <si>
-    <t>Rs. 1.85 Lakh</t>
-  </si>
-  <si>
-    <t>50 Used Kia Seltos</t>
-  </si>
-  <si>
-    <t>Rs. 3.69 Lakh</t>
-  </si>
-  <si>
-    <t>48 Used Hyundai Creta</t>
-  </si>
-  <si>
-    <t>Rs. 3.45 Lakh</t>
+    <t>Hyundai Grand i10 1.2 Kappa Asta</t>
+  </si>
+  <si>
+    <t>Rs. 3.18 Lakh</t>
+  </si>
+  <si>
+    <t>Hyundai i10 Magna 1.1</t>
+  </si>
+  <si>
+    <t>Rs. 3.05 Lakh</t>
+  </si>
+  <si>
+    <t>41 Used Hyundai Creta</t>
+  </si>
+  <si>
+    <t>Rs. 3.79 Lakh</t>
   </si>
 </sst>
 </file>
@@ -282,7 +270,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <sheetData>
     <row r="1">
@@ -317,22 +305,6 @@
         <v>30</v>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="s" s="0">
-        <v>31</v>
-      </c>
-      <c r="B5" t="s" s="0">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="s" s="0">
-        <v>33</v>
-      </c>
-      <c r="B6" t="s" s="0">
-        <v>34</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>

</xml_diff>

<commit_message>
Final Proj before First Review
</commit_message>
<xml_diff>
--- a/src/test/resources/testdata/Vehicle.xlsx
+++ b/src/test/resources/testdata/Vehicle.xlsx
@@ -8,12 +8,14 @@
   <sheets>
     <sheet name="HondaBikesUnder4Lakhs" r:id="rId3" sheetId="1"/>
     <sheet name="CarsUnder4Lakh" r:id="rId4" sheetId="2"/>
+    <sheet name="HondaBikes" r:id="rId5" sheetId="3"/>
+    <sheet name="HyundaiPopularCars" r:id="rId6" sheetId="4"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="80">
   <si>
     <t>Bike Name</t>
   </si>
@@ -106,6 +108,153 @@
   </si>
   <si>
     <t>Rs. 3.79 Lakh</t>
+  </si>
+  <si>
+    <t>ALL HONDA BIKE DETAILS</t>
+  </si>
+  <si>
+    <t>Honda CBR500R</t>
+  </si>
+  <si>
+    <t>Rs. 5.50 Lakh</t>
+  </si>
+  <si>
+    <t>Expected Launch : Jan 2028</t>
+  </si>
+  <si>
+    <t>Honda Rebel 1100</t>
+  </si>
+  <si>
+    <t>Rs. 12.00 Lakh</t>
+  </si>
+  <si>
+    <t>Honda CB500F</t>
+  </si>
+  <si>
+    <t>Rs. 5.00 Lakh</t>
+  </si>
+  <si>
+    <t>Honda Activa 7G</t>
+  </si>
+  <si>
+    <t>Rs. 14.46 Lakh</t>
+  </si>
+  <si>
+    <t>Honda CB1000R</t>
+  </si>
+  <si>
+    <t>Rs. 6.00 Lakh</t>
+  </si>
+  <si>
+    <t>Honda CB1000GT</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>Honda WN7</t>
+  </si>
+  <si>
+    <t>Honda SH125i</t>
+  </si>
+  <si>
+    <t>Honda CL500 Scrambler</t>
+  </si>
+  <si>
+    <t>HYUNDAI POPULAR CARS - CHENNAI</t>
+  </si>
+  <si>
+    <t>Car Price</t>
+  </si>
+  <si>
+    <t>Honda Amaze VX</t>
+  </si>
+  <si>
+    <t>Rs. 8.50 Lakh</t>
+  </si>
+  <si>
+    <t>Honda City i VTEC CVT VX</t>
+  </si>
+  <si>
+    <t>Rs. 3.99 Lakh</t>
+  </si>
+  <si>
+    <t>Honda City i-DTEC ZX</t>
+  </si>
+  <si>
+    <t>Rs. 10.50 Lakh</t>
+  </si>
+  <si>
+    <t>Honda City 1.5 S AT</t>
+  </si>
+  <si>
+    <t>Rs. 3.85 Lakh</t>
+  </si>
+  <si>
+    <t>Honda City V MT</t>
+  </si>
+  <si>
+    <t>Rs. 9.75 Lakh</t>
+  </si>
+  <si>
+    <t>Honda Amaze S Petrol BSIV</t>
+  </si>
+  <si>
+    <t>39 Used Maruti Swift</t>
+  </si>
+  <si>
+    <t>Rs. 3.65 Lakh</t>
+  </si>
+  <si>
+    <t>36 Used Hyundai Creta</t>
+  </si>
+  <si>
+    <t>Rs. 1.10 Lakh</t>
+  </si>
+  <si>
+    <t>31 Used Maruti Wagon R</t>
+  </si>
+  <si>
+    <t>Rs. 4.25 Lakh</t>
+  </si>
+  <si>
+    <t>53 Used Hyundai i20</t>
+  </si>
+  <si>
+    <t>Rs. 2.50 Lakh</t>
+  </si>
+  <si>
+    <t>1355 Used Maruti Alto 800</t>
+  </si>
+  <si>
+    <t>Rs. 5.69 Lakh</t>
+  </si>
+  <si>
+    <t>1330 Used Maruti Baleno</t>
+  </si>
+  <si>
+    <t>Rs. 1.56 Lakh</t>
+  </si>
+  <si>
+    <t>1234 Used Maruti Swift Dzire</t>
+  </si>
+  <si>
+    <t>1213 Used Tata Nexon</t>
+  </si>
+  <si>
+    <t>33 Used Hyundai Grand i10</t>
+  </si>
+  <si>
+    <t>Honda Amaze VX i-VTEC</t>
+  </si>
+  <si>
+    <t>Honda City 1.5 V AT</t>
+  </si>
+  <si>
+    <t>Honda Jazz ZX CVT</t>
+  </si>
+  <si>
+    <t>Honda City S</t>
   </si>
 </sst>
 </file>
@@ -308,4 +457,419 @@
   </sheetData>
   <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:C20"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s" s="0">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>3</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s" s="0">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>6</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>7</v>
+      </c>
+      <c r="C4" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>32</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>33</v>
+      </c>
+      <c r="C5" t="s" s="0">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>9</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>10</v>
+      </c>
+      <c r="C6" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>35</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>37</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>38</v>
+      </c>
+      <c r="C8" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>11</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>12</v>
+      </c>
+      <c r="C9" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>14</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="C10" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>16</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>17</v>
+      </c>
+      <c r="C11" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>18</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>19</v>
+      </c>
+      <c r="C12" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>20</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>15</v>
+      </c>
+      <c r="C13" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>21</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>22</v>
+      </c>
+      <c r="C14" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>39</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>40</v>
+      </c>
+      <c r="C15" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>41</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>42</v>
+      </c>
+      <c r="C16" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>43</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="C17" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>45</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="C18" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>46</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="C19" t="s" s="0">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>47</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>44</v>
+      </c>
+      <c r="C20" t="s" s="0">
+        <v>8</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <dimension ref="A1:B23"/>
+  <sheetFormatPr defaultRowHeight="15.0"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="s" s="0">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="s" s="0">
+        <v>23</v>
+      </c>
+      <c r="B2" t="s" s="0">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="s" s="0">
+        <v>50</v>
+      </c>
+      <c r="B3" t="s" s="0">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="B4" t="s" s="0">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="s" s="0">
+        <v>54</v>
+      </c>
+      <c r="B5" t="s" s="0">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="s" s="0">
+        <v>56</v>
+      </c>
+      <c r="B6" t="s" s="0">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="B7" t="s" s="0">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="s" s="0">
+        <v>60</v>
+      </c>
+      <c r="B8" t="s" s="0">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="s" s="0">
+        <v>61</v>
+      </c>
+      <c r="B9" t="s" s="0">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="s" s="0">
+        <v>63</v>
+      </c>
+      <c r="B10" t="s" s="0">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="s" s="0">
+        <v>65</v>
+      </c>
+      <c r="B11" t="s" s="0">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="s" s="0">
+        <v>67</v>
+      </c>
+      <c r="B12" t="s" s="0">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="s" s="0">
+        <v>69</v>
+      </c>
+      <c r="B13" t="s" s="0">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="s" s="0">
+        <v>71</v>
+      </c>
+      <c r="B14" t="s" s="0">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="s" s="0">
+        <v>73</v>
+      </c>
+      <c r="B15" t="s" s="0">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="s" s="0">
+        <v>74</v>
+      </c>
+      <c r="B16" t="s" s="0">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="0">
+        <v>75</v>
+      </c>
+      <c r="B17" t="s" s="0">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="0">
+        <v>76</v>
+      </c>
+      <c r="B18" t="s" s="0">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="0">
+        <v>58</v>
+      </c>
+      <c r="B19" t="s" s="0">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="0">
+        <v>52</v>
+      </c>
+      <c r="B20" t="s" s="0">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="0">
+        <v>77</v>
+      </c>
+      <c r="B21" t="s" s="0">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="0">
+        <v>78</v>
+      </c>
+      <c r="B22" t="s" s="0">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s" s="0">
+        <v>79</v>
+      </c>
+      <c r="B23" t="s" s="0">
+        <v>44</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins bottom="0.75" footer="0.3" header="0.3" left="0.7" right="0.7" top="0.75"/>
+</worksheet>
 </file>
</xml_diff>